<commit_message>
Etappe 5: Strategienamen auf den Folien stimmig, Umbenennung wird gemeldet
Die Wertentwicklungs-Folie bekam ihren Titel aus dem Mapping, die
Struktur-Folie davor traegt ihn fest aus der Vorlage. In cVV, ESG, ETF und
comdirect hiess dieselbe Strategie so auf zwei Folien hintereinander
verschieden ("ESG Defensiv Plus" / "ESG defensiv+").

- pptx_slides.strategiename_aus_titel: Wertentwicklungs-Folie uebernimmt
  den Namen der Struktur-Folie (feste Bloecke)
- Mapping_Strategien.xlsx: comdirect-Kasten "Portfolioverwaltung 30/70/100"
  statt "FFPB Strategie ..." (nur sheet1.xml, drei Zellen)
- chart_dynamik: tote Eintraege "comdirect 30/70/100" entfernt,
  _familie_aus_text herausgeloest
- tests/test_namen_folien.py (40. Suite) mit Kochrezept fuer Umbenennungen;
  gegen den alten Code rot
- STATUS, CLAUDE, PROJEKT_DOKUMENTATION nachgezogen

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mapping_Strategien.xlsx
+++ b/Mapping_Strategien.xlsx
@@ -1242,7 +1242,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>FFPB Strategie 30</t>
+          <t>Portfolioverwaltung 30</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>FFPB Strategie 70</t>
+          <t>Portfolioverwaltung 70</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>FFPB Strategie 100</t>
+          <t>Portfolioverwaltung 100</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">

</xml_diff>